<commit_message>
Bulk email import: one draft per row with downloadable templates
Add downloadable .xlsx/.csv import templates and create one draft per
row on import. New column format: name, company, email, subject, message,
with {{name}}/{{company}}/{{email}} placeholders filled per row.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/bulk-email-template.xlsx
+++ b/public/bulk-email-template.xlsx
@@ -397,121 +397,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="36.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>company</v>
+      </c>
+      <c r="C1" t="str">
         <v>email</v>
       </c>
-      <c r="B1" t="str">
-        <v>full_name</v>
-      </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>subject</v>
       </c>
-      <c r="D1" t="str">
-        <v>body</v>
+      <c r="E1" t="str">
+        <v>message</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>alice.smith@example.com</v>
+        <v>Jane Doe</v>
       </c>
       <c r="B2" t="str">
-        <v>Alice Smith</v>
+        <v>Acme Inc</v>
       </c>
       <c r="C2" t="str">
-        <v>Quick intro — {{full_name}}</v>
-      </c>
-      <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {{full_name}},
-I wanted to reach out to introduce our latest offer.
-Looking forward to connecting!
-Best regards,
+        <v>jane.doe@example.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Quick question, {{name}}</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {{name}},
+I wanted to reach out to {{company}} regarding...
+Best,
 Your Name</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>bob.jones@company.io</v>
+        <v>John Smith</v>
       </c>
       <c r="B3" t="str">
-        <v>Bob Jones</v>
+        <v>Globex</v>
       </c>
       <c r="C3" t="str">
-        <v>Quick intro — {{full_name}}</v>
-      </c>
-      <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {{full_name}},
-I wanted to reach out to introduce our latest offer.
-Looking forward to connecting!
-Best regards,
-Your Name</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>carol.white@startup.co</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Carol White</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Quick intro — {{full_name}}</v>
-      </c>
-      <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {{full_name}},
-I wanted to reach out to introduce our latest offer.
-Looking forward to connecting!
-Best regards,
-Your Name</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>david.brown@corp.com</v>
-      </c>
-      <c r="B5" t="str">
-        <v>David Brown</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Quick intro — {{full_name}}</v>
-      </c>
-      <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {{full_name}},
-I wanted to reach out to introduce our latest offer.
-Looking forward to connecting!
-Best regards,
-Your Name</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>eva.green@agency.net</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Eva Green</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Quick intro — {{full_name}}</v>
-      </c>
-      <c r="D6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {{full_name}},
-I wanted to reach out to introduce our latest offer.
-Looking forward to connecting!
-Best regards,
+        <v>john.smith@example.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Following up with {{company}}</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {{name}},
+Just circling back...
+Best,
 Your Name</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>